<commit_message>
Show Data Paint and Welding for QA/QC tab
</commit_message>
<xml_diff>
--- a/MPR_Managerment/Templates/material_receiving_inspection_report__material_template.xlsx
+++ b/MPR_Managerment/Templates/material_receiving_inspection_report__material_template.xlsx
@@ -1036,8 +1036,221 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="54" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="54" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="55" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="54" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="8" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="49" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1048,15 +1261,48 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="32" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="15" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="15" fontId="8" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1072,13 +1318,16 @@
     <xf numFmtId="14" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1091,6 +1340,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1123,6 +1375,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1131,261 +1386,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="32" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="8" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="49" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="54" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="54" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="54" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="55" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1523,7 +1523,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="#REF!" spid="_x0000_s7588"/>
+                  <a14:cameraTool cellRange="#REF!" spid="_x0000_s7589"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1912,462 +1912,462 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:140" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="69"/>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="78" t="s">
+      <c r="A1" s="27"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
-      <c r="L1" s="79"/>
-      <c r="M1" s="79"/>
-      <c r="N1" s="79"/>
-      <c r="O1" s="79"/>
-      <c r="P1" s="79"/>
-      <c r="Q1" s="79"/>
-      <c r="R1" s="79"/>
-      <c r="S1" s="79"/>
-      <c r="T1" s="79"/>
-      <c r="U1" s="79"/>
-      <c r="V1" s="79"/>
-      <c r="W1" s="79"/>
-      <c r="X1" s="79"/>
-      <c r="Y1" s="79"/>
-      <c r="Z1" s="79"/>
-      <c r="AA1" s="79"/>
-      <c r="AB1" s="79"/>
-      <c r="AC1" s="79"/>
-      <c r="AD1" s="79"/>
-      <c r="AE1" s="79"/>
-      <c r="AF1" s="79"/>
-      <c r="AG1" s="79"/>
-      <c r="AH1" s="79"/>
-      <c r="AI1" s="79"/>
-      <c r="AJ1" s="79"/>
-      <c r="AK1" s="79"/>
-      <c r="AL1" s="86" t="s">
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+      <c r="P1" s="37"/>
+      <c r="Q1" s="37"/>
+      <c r="R1" s="37"/>
+      <c r="S1" s="37"/>
+      <c r="T1" s="37"/>
+      <c r="U1" s="37"/>
+      <c r="V1" s="37"/>
+      <c r="W1" s="37"/>
+      <c r="X1" s="37"/>
+      <c r="Y1" s="37"/>
+      <c r="Z1" s="37"/>
+      <c r="AA1" s="37"/>
+      <c r="AB1" s="37"/>
+      <c r="AC1" s="37"/>
+      <c r="AD1" s="37"/>
+      <c r="AE1" s="37"/>
+      <c r="AF1" s="37"/>
+      <c r="AG1" s="37"/>
+      <c r="AH1" s="37"/>
+      <c r="AI1" s="37"/>
+      <c r="AJ1" s="37"/>
+      <c r="AK1" s="37"/>
+      <c r="AL1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="AM1" s="87"/>
-      <c r="AN1" s="87"/>
-      <c r="AO1" s="87"/>
-      <c r="AP1" s="87"/>
-      <c r="AQ1" s="87"/>
-      <c r="AR1" s="88"/>
-      <c r="AS1" s="89" t="s">
+      <c r="AM1" s="45"/>
+      <c r="AN1" s="45"/>
+      <c r="AO1" s="45"/>
+      <c r="AP1" s="45"/>
+      <c r="AQ1" s="45"/>
+      <c r="AR1" s="46"/>
+      <c r="AS1" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="AT1" s="89"/>
-      <c r="AU1" s="89"/>
-      <c r="AV1" s="90"/>
+      <c r="AT1" s="47"/>
+      <c r="AU1" s="47"/>
+      <c r="AV1" s="48"/>
     </row>
     <row r="2" spans="1:140" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="72"/>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="74"/>
-      <c r="I2" s="80"/>
-      <c r="J2" s="81"/>
-      <c r="K2" s="81"/>
-      <c r="L2" s="81"/>
-      <c r="M2" s="81"/>
-      <c r="N2" s="81"/>
-      <c r="O2" s="81"/>
-      <c r="P2" s="81"/>
-      <c r="Q2" s="81"/>
-      <c r="R2" s="81"/>
-      <c r="S2" s="81"/>
-      <c r="T2" s="81"/>
-      <c r="U2" s="81"/>
-      <c r="V2" s="81"/>
-      <c r="W2" s="81"/>
-      <c r="X2" s="81"/>
-      <c r="Y2" s="81"/>
-      <c r="Z2" s="81"/>
-      <c r="AA2" s="81"/>
-      <c r="AB2" s="81"/>
-      <c r="AC2" s="81"/>
-      <c r="AD2" s="81"/>
-      <c r="AE2" s="81"/>
-      <c r="AF2" s="81"/>
-      <c r="AG2" s="81"/>
-      <c r="AH2" s="81"/>
-      <c r="AI2" s="81"/>
-      <c r="AJ2" s="81"/>
-      <c r="AK2" s="81"/>
-      <c r="AL2" s="91" t="s">
+      <c r="A2" s="30"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="38"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="39"/>
+      <c r="M2" s="39"/>
+      <c r="N2" s="39"/>
+      <c r="O2" s="39"/>
+      <c r="P2" s="39"/>
+      <c r="Q2" s="39"/>
+      <c r="R2" s="39"/>
+      <c r="S2" s="39"/>
+      <c r="T2" s="39"/>
+      <c r="U2" s="39"/>
+      <c r="V2" s="39"/>
+      <c r="W2" s="39"/>
+      <c r="X2" s="39"/>
+      <c r="Y2" s="39"/>
+      <c r="Z2" s="39"/>
+      <c r="AA2" s="39"/>
+      <c r="AB2" s="39"/>
+      <c r="AC2" s="39"/>
+      <c r="AD2" s="39"/>
+      <c r="AE2" s="39"/>
+      <c r="AF2" s="39"/>
+      <c r="AG2" s="39"/>
+      <c r="AH2" s="39"/>
+      <c r="AI2" s="39"/>
+      <c r="AJ2" s="39"/>
+      <c r="AK2" s="39"/>
+      <c r="AL2" s="49" t="s">
         <v>3</v>
       </c>
-      <c r="AM2" s="92"/>
-      <c r="AN2" s="92"/>
-      <c r="AO2" s="92"/>
-      <c r="AP2" s="92"/>
-      <c r="AQ2" s="92"/>
-      <c r="AR2" s="93"/>
-      <c r="AS2" s="94" t="s">
+      <c r="AM2" s="50"/>
+      <c r="AN2" s="50"/>
+      <c r="AO2" s="50"/>
+      <c r="AP2" s="50"/>
+      <c r="AQ2" s="50"/>
+      <c r="AR2" s="51"/>
+      <c r="AS2" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="AT2" s="95"/>
-      <c r="AU2" s="95"/>
-      <c r="AV2" s="96"/>
+      <c r="AT2" s="53"/>
+      <c r="AU2" s="53"/>
+      <c r="AV2" s="54"/>
     </row>
     <row r="3" spans="1:140" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="72"/>
-      <c r="B3" s="73"/>
-      <c r="C3" s="73"/>
-      <c r="D3" s="73"/>
-      <c r="E3" s="73"/>
-      <c r="F3" s="73"/>
-      <c r="G3" s="73"/>
-      <c r="H3" s="74"/>
-      <c r="I3" s="80"/>
-      <c r="J3" s="81"/>
-      <c r="K3" s="81"/>
-      <c r="L3" s="81"/>
-      <c r="M3" s="81"/>
-      <c r="N3" s="81"/>
-      <c r="O3" s="81"/>
-      <c r="P3" s="81"/>
-      <c r="Q3" s="81"/>
-      <c r="R3" s="81"/>
-      <c r="S3" s="81"/>
-      <c r="T3" s="81"/>
-      <c r="U3" s="81"/>
-      <c r="V3" s="81"/>
-      <c r="W3" s="81"/>
-      <c r="X3" s="81"/>
-      <c r="Y3" s="81"/>
-      <c r="Z3" s="81"/>
-      <c r="AA3" s="81"/>
-      <c r="AB3" s="81"/>
-      <c r="AC3" s="81"/>
-      <c r="AD3" s="81"/>
-      <c r="AE3" s="81"/>
-      <c r="AF3" s="81"/>
-      <c r="AG3" s="81"/>
-      <c r="AH3" s="81"/>
-      <c r="AI3" s="81"/>
-      <c r="AJ3" s="81"/>
-      <c r="AK3" s="81"/>
-      <c r="AL3" s="97" t="s">
+      <c r="A3" s="30"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="38"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="39"/>
+      <c r="L3" s="39"/>
+      <c r="M3" s="39"/>
+      <c r="N3" s="39"/>
+      <c r="O3" s="39"/>
+      <c r="P3" s="39"/>
+      <c r="Q3" s="39"/>
+      <c r="R3" s="39"/>
+      <c r="S3" s="39"/>
+      <c r="T3" s="39"/>
+      <c r="U3" s="39"/>
+      <c r="V3" s="39"/>
+      <c r="W3" s="39"/>
+      <c r="X3" s="39"/>
+      <c r="Y3" s="39"/>
+      <c r="Z3" s="39"/>
+      <c r="AA3" s="39"/>
+      <c r="AB3" s="39"/>
+      <c r="AC3" s="39"/>
+      <c r="AD3" s="39"/>
+      <c r="AE3" s="39"/>
+      <c r="AF3" s="39"/>
+      <c r="AG3" s="39"/>
+      <c r="AH3" s="39"/>
+      <c r="AI3" s="39"/>
+      <c r="AJ3" s="39"/>
+      <c r="AK3" s="39"/>
+      <c r="AL3" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="AM3" s="98"/>
-      <c r="AN3" s="98"/>
-      <c r="AO3" s="98"/>
-      <c r="AP3" s="98"/>
-      <c r="AQ3" s="98"/>
-      <c r="AR3" s="99"/>
-      <c r="AS3" s="100">
+      <c r="AM3" s="56"/>
+      <c r="AN3" s="56"/>
+      <c r="AO3" s="56"/>
+      <c r="AP3" s="56"/>
+      <c r="AQ3" s="56"/>
+      <c r="AR3" s="57"/>
+      <c r="AS3" s="58">
         <v>44761</v>
       </c>
-      <c r="AT3" s="101"/>
-      <c r="AU3" s="101"/>
-      <c r="AV3" s="102"/>
+      <c r="AT3" s="59"/>
+      <c r="AU3" s="59"/>
+      <c r="AV3" s="60"/>
     </row>
     <row r="4" spans="1:140" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="72"/>
-      <c r="B4" s="73"/>
-      <c r="C4" s="73"/>
-      <c r="D4" s="73"/>
-      <c r="E4" s="73"/>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
-      <c r="H4" s="74"/>
-      <c r="I4" s="80"/>
-      <c r="J4" s="81"/>
-      <c r="K4" s="81"/>
-      <c r="L4" s="81"/>
-      <c r="M4" s="81"/>
-      <c r="N4" s="81"/>
-      <c r="O4" s="81"/>
-      <c r="P4" s="81"/>
-      <c r="Q4" s="81"/>
-      <c r="R4" s="81"/>
-      <c r="S4" s="81"/>
-      <c r="T4" s="81"/>
-      <c r="U4" s="81"/>
-      <c r="V4" s="81"/>
-      <c r="W4" s="81"/>
-      <c r="X4" s="81"/>
-      <c r="Y4" s="81"/>
-      <c r="Z4" s="81"/>
-      <c r="AA4" s="81"/>
-      <c r="AB4" s="81"/>
-      <c r="AC4" s="81"/>
-      <c r="AD4" s="81"/>
-      <c r="AE4" s="81"/>
-      <c r="AF4" s="81"/>
-      <c r="AG4" s="81"/>
-      <c r="AH4" s="81"/>
-      <c r="AI4" s="81"/>
-      <c r="AJ4" s="81"/>
-      <c r="AK4" s="82"/>
-      <c r="AL4" s="103" t="s">
+      <c r="A4" s="30"/>
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="38"/>
+      <c r="J4" s="39"/>
+      <c r="K4" s="39"/>
+      <c r="L4" s="39"/>
+      <c r="M4" s="39"/>
+      <c r="N4" s="39"/>
+      <c r="O4" s="39"/>
+      <c r="P4" s="39"/>
+      <c r="Q4" s="39"/>
+      <c r="R4" s="39"/>
+      <c r="S4" s="39"/>
+      <c r="T4" s="39"/>
+      <c r="U4" s="39"/>
+      <c r="V4" s="39"/>
+      <c r="W4" s="39"/>
+      <c r="X4" s="39"/>
+      <c r="Y4" s="39"/>
+      <c r="Z4" s="39"/>
+      <c r="AA4" s="39"/>
+      <c r="AB4" s="39"/>
+      <c r="AC4" s="39"/>
+      <c r="AD4" s="39"/>
+      <c r="AE4" s="39"/>
+      <c r="AF4" s="39"/>
+      <c r="AG4" s="39"/>
+      <c r="AH4" s="39"/>
+      <c r="AI4" s="39"/>
+      <c r="AJ4" s="39"/>
+      <c r="AK4" s="40"/>
+      <c r="AL4" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="AM4" s="104"/>
-      <c r="AN4" s="104"/>
-      <c r="AO4" s="104"/>
-      <c r="AP4" s="104"/>
-      <c r="AQ4" s="104"/>
-      <c r="AR4" s="104"/>
-      <c r="AS4" s="105"/>
-      <c r="AT4" s="105"/>
-      <c r="AU4" s="105"/>
-      <c r="AV4" s="106"/>
+      <c r="AM4" s="62"/>
+      <c r="AN4" s="62"/>
+      <c r="AO4" s="62"/>
+      <c r="AP4" s="62"/>
+      <c r="AQ4" s="62"/>
+      <c r="AR4" s="62"/>
+      <c r="AS4" s="63"/>
+      <c r="AT4" s="63"/>
+      <c r="AU4" s="63"/>
+      <c r="AV4" s="64"/>
     </row>
     <row r="5" spans="1:140" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="75"/>
-      <c r="B5" s="76"/>
-      <c r="C5" s="76"/>
-      <c r="D5" s="76"/>
-      <c r="E5" s="76"/>
-      <c r="F5" s="76"/>
-      <c r="G5" s="76"/>
-      <c r="H5" s="77"/>
-      <c r="I5" s="83"/>
-      <c r="J5" s="84"/>
-      <c r="K5" s="84"/>
-      <c r="L5" s="84"/>
-      <c r="M5" s="84"/>
-      <c r="N5" s="84"/>
-      <c r="O5" s="84"/>
-      <c r="P5" s="84"/>
-      <c r="Q5" s="84"/>
-      <c r="R5" s="84"/>
-      <c r="S5" s="84"/>
-      <c r="T5" s="84"/>
-      <c r="U5" s="84"/>
-      <c r="V5" s="84"/>
-      <c r="W5" s="84"/>
-      <c r="X5" s="84"/>
-      <c r="Y5" s="84"/>
-      <c r="Z5" s="84"/>
-      <c r="AA5" s="84"/>
-      <c r="AB5" s="84"/>
-      <c r="AC5" s="84"/>
-      <c r="AD5" s="84"/>
-      <c r="AE5" s="84"/>
-      <c r="AF5" s="84"/>
-      <c r="AG5" s="84"/>
-      <c r="AH5" s="84"/>
-      <c r="AI5" s="84"/>
-      <c r="AJ5" s="84"/>
-      <c r="AK5" s="85"/>
-      <c r="AL5" s="107" t="s">
+      <c r="A5" s="33"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="42"/>
+      <c r="L5" s="42"/>
+      <c r="M5" s="42"/>
+      <c r="N5" s="42"/>
+      <c r="O5" s="42"/>
+      <c r="P5" s="42"/>
+      <c r="Q5" s="42"/>
+      <c r="R5" s="42"/>
+      <c r="S5" s="42"/>
+      <c r="T5" s="42"/>
+      <c r="U5" s="42"/>
+      <c r="V5" s="42"/>
+      <c r="W5" s="42"/>
+      <c r="X5" s="42"/>
+      <c r="Y5" s="42"/>
+      <c r="Z5" s="42"/>
+      <c r="AA5" s="42"/>
+      <c r="AB5" s="42"/>
+      <c r="AC5" s="42"/>
+      <c r="AD5" s="42"/>
+      <c r="AE5" s="42"/>
+      <c r="AF5" s="42"/>
+      <c r="AG5" s="42"/>
+      <c r="AH5" s="42"/>
+      <c r="AI5" s="42"/>
+      <c r="AJ5" s="42"/>
+      <c r="AK5" s="43"/>
+      <c r="AL5" s="65" t="s">
         <v>6</v>
       </c>
-      <c r="AM5" s="108"/>
-      <c r="AN5" s="108"/>
-      <c r="AO5" s="108"/>
-      <c r="AP5" s="108"/>
-      <c r="AQ5" s="108"/>
-      <c r="AR5" s="108"/>
-      <c r="AS5" s="109"/>
-      <c r="AT5" s="110"/>
-      <c r="AU5" s="110"/>
-      <c r="AV5" s="111"/>
+      <c r="AM5" s="66"/>
+      <c r="AN5" s="66"/>
+      <c r="AO5" s="66"/>
+      <c r="AP5" s="66"/>
+      <c r="AQ5" s="66"/>
+      <c r="AR5" s="66"/>
+      <c r="AS5" s="67"/>
+      <c r="AT5" s="68"/>
+      <c r="AU5" s="68"/>
+      <c r="AV5" s="69"/>
     </row>
     <row r="6" spans="1:140" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="65" t="s">
+      <c r="A6" s="73" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="66"/>
-      <c r="C6" s="66"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
-      <c r="G6" s="55" t="s">
+      <c r="B6" s="74"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="74"/>
+      <c r="G6" s="75" t="s">
         <v>42</v>
       </c>
-      <c r="H6" s="55"/>
-      <c r="I6" s="67"/>
-      <c r="J6" s="67"/>
-      <c r="K6" s="67"/>
-      <c r="L6" s="67"/>
-      <c r="M6" s="67"/>
-      <c r="N6" s="67"/>
-      <c r="O6" s="67"/>
-      <c r="P6" s="67"/>
-      <c r="Q6" s="68" t="s">
+      <c r="H6" s="75"/>
+      <c r="I6" s="76"/>
+      <c r="J6" s="76"/>
+      <c r="K6" s="76"/>
+      <c r="L6" s="76"/>
+      <c r="M6" s="76"/>
+      <c r="N6" s="76"/>
+      <c r="O6" s="76"/>
+      <c r="P6" s="76"/>
+      <c r="Q6" s="77" t="s">
         <v>7</v>
       </c>
-      <c r="R6" s="68"/>
-      <c r="S6" s="68"/>
-      <c r="T6" s="68"/>
-      <c r="U6" s="68"/>
-      <c r="V6" s="68"/>
-      <c r="W6" s="67" t="s">
+      <c r="R6" s="77"/>
+      <c r="S6" s="77"/>
+      <c r="T6" s="77"/>
+      <c r="U6" s="77"/>
+      <c r="V6" s="77"/>
+      <c r="W6" s="76" t="s">
         <v>39</v>
       </c>
-      <c r="X6" s="67"/>
-      <c r="Y6" s="67"/>
-      <c r="Z6" s="67"/>
-      <c r="AA6" s="67"/>
-      <c r="AB6" s="67"/>
-      <c r="AC6" s="67"/>
-      <c r="AD6" s="67"/>
-      <c r="AE6" s="67"/>
-      <c r="AF6" s="67"/>
-      <c r="AG6" s="68" t="s">
+      <c r="X6" s="76"/>
+      <c r="Y6" s="76"/>
+      <c r="Z6" s="76"/>
+      <c r="AA6" s="76"/>
+      <c r="AB6" s="76"/>
+      <c r="AC6" s="76"/>
+      <c r="AD6" s="76"/>
+      <c r="AE6" s="76"/>
+      <c r="AF6" s="76"/>
+      <c r="AG6" s="77" t="s">
         <v>8</v>
       </c>
-      <c r="AH6" s="68"/>
-      <c r="AI6" s="68"/>
-      <c r="AJ6" s="68"/>
-      <c r="AK6" s="68"/>
-      <c r="AL6" s="55" t="s">
+      <c r="AH6" s="77"/>
+      <c r="AI6" s="77"/>
+      <c r="AJ6" s="77"/>
+      <c r="AK6" s="77"/>
+      <c r="AL6" s="75" t="s">
         <v>40</v>
       </c>
-      <c r="AM6" s="55"/>
-      <c r="AN6" s="55"/>
-      <c r="AO6" s="55"/>
-      <c r="AP6" s="55"/>
-      <c r="AQ6" s="55"/>
-      <c r="AR6" s="55"/>
-      <c r="AS6" s="55"/>
-      <c r="AT6" s="55"/>
-      <c r="AU6" s="55"/>
-      <c r="AV6" s="56"/>
+      <c r="AM6" s="75"/>
+      <c r="AN6" s="75"/>
+      <c r="AO6" s="75"/>
+      <c r="AP6" s="75"/>
+      <c r="AQ6" s="75"/>
+      <c r="AR6" s="75"/>
+      <c r="AS6" s="75"/>
+      <c r="AT6" s="75"/>
+      <c r="AU6" s="75"/>
+      <c r="AV6" s="83"/>
     </row>
     <row r="7" spans="1:140" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="112" t="s">
+      <c r="A7" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="113"/>
-      <c r="C7" s="113"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="114" t="s">
+      <c r="B7" s="79"/>
+      <c r="C7" s="79"/>
+      <c r="D7" s="79"/>
+      <c r="E7" s="79"/>
+      <c r="F7" s="79"/>
+      <c r="G7" s="80" t="s">
         <v>41</v>
       </c>
-      <c r="H7" s="115"/>
-      <c r="I7" s="115"/>
-      <c r="J7" s="115"/>
-      <c r="K7" s="115"/>
-      <c r="L7" s="115"/>
-      <c r="M7" s="115"/>
-      <c r="N7" s="115"/>
-      <c r="O7" s="115"/>
-      <c r="P7" s="115"/>
-      <c r="Q7" s="113" t="s">
+      <c r="H7" s="81"/>
+      <c r="I7" s="81"/>
+      <c r="J7" s="81"/>
+      <c r="K7" s="81"/>
+      <c r="L7" s="81"/>
+      <c r="M7" s="81"/>
+      <c r="N7" s="81"/>
+      <c r="O7" s="81"/>
+      <c r="P7" s="81"/>
+      <c r="Q7" s="79" t="s">
         <v>34</v>
       </c>
-      <c r="R7" s="113"/>
-      <c r="S7" s="113"/>
-      <c r="T7" s="113"/>
-      <c r="U7" s="113"/>
-      <c r="V7" s="113"/>
-      <c r="W7" s="116"/>
-      <c r="X7" s="115"/>
-      <c r="Y7" s="115"/>
-      <c r="Z7" s="115"/>
-      <c r="AA7" s="115"/>
-      <c r="AB7" s="115"/>
-      <c r="AC7" s="115"/>
-      <c r="AD7" s="115"/>
-      <c r="AE7" s="115"/>
-      <c r="AF7" s="115"/>
-      <c r="AG7" s="113" t="s">
+      <c r="R7" s="79"/>
+      <c r="S7" s="79"/>
+      <c r="T7" s="79"/>
+      <c r="U7" s="79"/>
+      <c r="V7" s="79"/>
+      <c r="W7" s="82"/>
+      <c r="X7" s="81"/>
+      <c r="Y7" s="81"/>
+      <c r="Z7" s="81"/>
+      <c r="AA7" s="81"/>
+      <c r="AB7" s="81"/>
+      <c r="AC7" s="81"/>
+      <c r="AD7" s="81"/>
+      <c r="AE7" s="81"/>
+      <c r="AF7" s="81"/>
+      <c r="AG7" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="AH7" s="113"/>
-      <c r="AI7" s="113"/>
-      <c r="AJ7" s="113"/>
-      <c r="AK7" s="113"/>
-      <c r="AL7" s="63" t="s">
+      <c r="AH7" s="79"/>
+      <c r="AI7" s="79"/>
+      <c r="AJ7" s="79"/>
+      <c r="AK7" s="79"/>
+      <c r="AL7" s="71" t="s">
         <v>43</v>
       </c>
-      <c r="AM7" s="63"/>
-      <c r="AN7" s="63"/>
-      <c r="AO7" s="63"/>
-      <c r="AP7" s="63"/>
-      <c r="AQ7" s="63"/>
-      <c r="AR7" s="63"/>
-      <c r="AS7" s="63"/>
-      <c r="AT7" s="63"/>
-      <c r="AU7" s="63"/>
-      <c r="AV7" s="64"/>
+      <c r="AM7" s="71"/>
+      <c r="AN7" s="71"/>
+      <c r="AO7" s="71"/>
+      <c r="AP7" s="71"/>
+      <c r="AQ7" s="71"/>
+      <c r="AR7" s="71"/>
+      <c r="AS7" s="71"/>
+      <c r="AT7" s="71"/>
+      <c r="AU7" s="71"/>
+      <c r="AV7" s="72"/>
     </row>
     <row r="8" spans="1:140" s="3" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="58" t="s">
+      <c r="A8" s="97" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="59"/>
-      <c r="C8" s="60" t="s">
+      <c r="B8" s="98"/>
+      <c r="C8" s="99" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="60"/>
-      <c r="G8" s="60"/>
-      <c r="H8" s="61" t="s">
+      <c r="D8" s="99"/>
+      <c r="E8" s="99"/>
+      <c r="F8" s="99"/>
+      <c r="G8" s="99"/>
+      <c r="H8" s="100" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="61"/>
-      <c r="J8" s="61"/>
-      <c r="K8" s="61"/>
-      <c r="L8" s="61"/>
-      <c r="M8" s="62" t="s">
+      <c r="I8" s="100"/>
+      <c r="J8" s="100"/>
+      <c r="K8" s="100"/>
+      <c r="L8" s="100"/>
+      <c r="M8" s="70" t="s">
         <v>33</v>
       </c>
-      <c r="N8" s="62"/>
-      <c r="O8" s="62"/>
-      <c r="P8" s="62"/>
-      <c r="Q8" s="62"/>
-      <c r="R8" s="62"/>
-      <c r="S8" s="62"/>
-      <c r="T8" s="57" t="s">
+      <c r="N8" s="70"/>
+      <c r="O8" s="70"/>
+      <c r="P8" s="70"/>
+      <c r="Q8" s="70"/>
+      <c r="R8" s="70"/>
+      <c r="S8" s="70"/>
+      <c r="T8" s="84" t="s">
         <v>13</v>
       </c>
-      <c r="U8" s="57"/>
-      <c r="V8" s="57"/>
-      <c r="W8" s="57" t="s">
+      <c r="U8" s="84"/>
+      <c r="V8" s="84"/>
+      <c r="W8" s="84" t="s">
         <v>14</v>
       </c>
-      <c r="X8" s="57"/>
-      <c r="Y8" s="61" t="s">
+      <c r="X8" s="84"/>
+      <c r="Y8" s="100" t="s">
         <v>28</v>
       </c>
-      <c r="Z8" s="61"/>
-      <c r="AA8" s="61"/>
-      <c r="AB8" s="61"/>
-      <c r="AC8" s="61"/>
-      <c r="AD8" s="61"/>
-      <c r="AE8" s="60" t="s">
+      <c r="Z8" s="100"/>
+      <c r="AA8" s="100"/>
+      <c r="AB8" s="100"/>
+      <c r="AC8" s="100"/>
+      <c r="AD8" s="100"/>
+      <c r="AE8" s="99" t="s">
         <v>15</v>
       </c>
-      <c r="AF8" s="60"/>
-      <c r="AG8" s="60"/>
-      <c r="AH8" s="60"/>
-      <c r="AI8" s="60"/>
-      <c r="AJ8" s="60"/>
-      <c r="AK8" s="60"/>
-      <c r="AL8" s="61" t="s">
+      <c r="AF8" s="99"/>
+      <c r="AG8" s="99"/>
+      <c r="AH8" s="99"/>
+      <c r="AI8" s="99"/>
+      <c r="AJ8" s="99"/>
+      <c r="AK8" s="99"/>
+      <c r="AL8" s="100" t="s">
         <v>16</v>
       </c>
-      <c r="AM8" s="61"/>
-      <c r="AN8" s="61"/>
-      <c r="AO8" s="61"/>
-      <c r="AP8" s="61"/>
-      <c r="AQ8" s="61"/>
-      <c r="AR8" s="61"/>
-      <c r="AS8" s="62" t="s">
+      <c r="AM8" s="100"/>
+      <c r="AN8" s="100"/>
+      <c r="AO8" s="100"/>
+      <c r="AP8" s="100"/>
+      <c r="AQ8" s="100"/>
+      <c r="AR8" s="100"/>
+      <c r="AS8" s="70" t="s">
         <v>30</v>
       </c>
-      <c r="AT8" s="62"/>
+      <c r="AT8" s="70"/>
       <c r="AU8" s="5" t="s">
         <v>31</v>
       </c>
@@ -2376,106 +2376,106 @@
       </c>
     </row>
     <row r="9" spans="1:140" s="3" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="126"/>
-      <c r="B9" s="120"/>
-      <c r="C9" s="121"/>
-      <c r="D9" s="121"/>
-      <c r="E9" s="121"/>
-      <c r="F9" s="121"/>
-      <c r="G9" s="121"/>
-      <c r="H9" s="122"/>
-      <c r="I9" s="122"/>
-      <c r="J9" s="122"/>
-      <c r="K9" s="122"/>
-      <c r="L9" s="122"/>
-      <c r="M9" s="123"/>
-      <c r="N9" s="123"/>
-      <c r="O9" s="123"/>
-      <c r="P9" s="123"/>
-      <c r="Q9" s="123"/>
-      <c r="R9" s="123"/>
-      <c r="S9" s="123"/>
-      <c r="T9" s="124"/>
-      <c r="U9" s="124"/>
-      <c r="V9" s="124"/>
-      <c r="W9" s="124"/>
-      <c r="X9" s="124"/>
-      <c r="Y9" s="122"/>
-      <c r="Z9" s="122"/>
-      <c r="AA9" s="122"/>
-      <c r="AB9" s="122"/>
-      <c r="AC9" s="122"/>
-      <c r="AD9" s="122"/>
-      <c r="AE9" s="121"/>
-      <c r="AF9" s="121"/>
-      <c r="AG9" s="121"/>
-      <c r="AH9" s="121"/>
-      <c r="AI9" s="121"/>
-      <c r="AJ9" s="121"/>
-      <c r="AK9" s="121"/>
-      <c r="AL9" s="122"/>
-      <c r="AM9" s="122"/>
-      <c r="AN9" s="122"/>
-      <c r="AO9" s="122"/>
-      <c r="AP9" s="122"/>
-      <c r="AQ9" s="122"/>
-      <c r="AR9" s="122"/>
-      <c r="AS9" s="123"/>
-      <c r="AT9" s="123"/>
-      <c r="AU9" s="125"/>
-      <c r="AV9" s="127"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="24"/>
+      <c r="N9" s="24"/>
+      <c r="O9" s="24"/>
+      <c r="P9" s="24"/>
+      <c r="Q9" s="24"/>
+      <c r="R9" s="24"/>
+      <c r="S9" s="24"/>
+      <c r="T9" s="21"/>
+      <c r="U9" s="21"/>
+      <c r="V9" s="21"/>
+      <c r="W9" s="21"/>
+      <c r="X9" s="21"/>
+      <c r="Y9" s="22"/>
+      <c r="Z9" s="22"/>
+      <c r="AA9" s="22"/>
+      <c r="AB9" s="22"/>
+      <c r="AC9" s="22"/>
+      <c r="AD9" s="22"/>
+      <c r="AE9" s="23"/>
+      <c r="AF9" s="23"/>
+      <c r="AG9" s="23"/>
+      <c r="AH9" s="23"/>
+      <c r="AI9" s="23"/>
+      <c r="AJ9" s="23"/>
+      <c r="AK9" s="23"/>
+      <c r="AL9" s="22"/>
+      <c r="AM9" s="22"/>
+      <c r="AN9" s="22"/>
+      <c r="AO9" s="22"/>
+      <c r="AP9" s="22"/>
+      <c r="AQ9" s="22"/>
+      <c r="AR9" s="22"/>
+      <c r="AS9" s="24"/>
+      <c r="AT9" s="24"/>
+      <c r="AU9" s="16"/>
+      <c r="AV9" s="17"/>
     </row>
     <row r="10" spans="1:140" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="117" t="s">
+      <c r="A10" s="85" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="118"/>
-      <c r="C10" s="118"/>
-      <c r="D10" s="118"/>
-      <c r="E10" s="118"/>
-      <c r="F10" s="118"/>
-      <c r="G10" s="118"/>
-      <c r="H10" s="118"/>
-      <c r="I10" s="118"/>
-      <c r="J10" s="118"/>
-      <c r="K10" s="118"/>
-      <c r="L10" s="118"/>
-      <c r="M10" s="118"/>
-      <c r="N10" s="118"/>
-      <c r="O10" s="118"/>
-      <c r="P10" s="118"/>
-      <c r="Q10" s="118"/>
-      <c r="R10" s="118"/>
-      <c r="S10" s="118"/>
-      <c r="T10" s="118"/>
-      <c r="U10" s="118"/>
-      <c r="V10" s="118"/>
-      <c r="W10" s="118"/>
-      <c r="X10" s="118"/>
-      <c r="Y10" s="118"/>
-      <c r="Z10" s="118"/>
-      <c r="AA10" s="118"/>
-      <c r="AB10" s="118"/>
-      <c r="AC10" s="118"/>
-      <c r="AD10" s="118"/>
-      <c r="AE10" s="118"/>
-      <c r="AF10" s="118"/>
-      <c r="AG10" s="118"/>
-      <c r="AH10" s="118"/>
-      <c r="AI10" s="118"/>
-      <c r="AJ10" s="118"/>
-      <c r="AK10" s="118"/>
-      <c r="AL10" s="118"/>
-      <c r="AM10" s="118"/>
-      <c r="AN10" s="118"/>
-      <c r="AO10" s="118"/>
-      <c r="AP10" s="118"/>
-      <c r="AQ10" s="118"/>
-      <c r="AR10" s="118"/>
-      <c r="AS10" s="118"/>
-      <c r="AT10" s="118"/>
-      <c r="AU10" s="118"/>
-      <c r="AV10" s="119"/>
+      <c r="B10" s="86"/>
+      <c r="C10" s="86"/>
+      <c r="D10" s="86"/>
+      <c r="E10" s="86"/>
+      <c r="F10" s="86"/>
+      <c r="G10" s="86"/>
+      <c r="H10" s="86"/>
+      <c r="I10" s="86"/>
+      <c r="J10" s="86"/>
+      <c r="K10" s="86"/>
+      <c r="L10" s="86"/>
+      <c r="M10" s="86"/>
+      <c r="N10" s="86"/>
+      <c r="O10" s="86"/>
+      <c r="P10" s="86"/>
+      <c r="Q10" s="86"/>
+      <c r="R10" s="86"/>
+      <c r="S10" s="86"/>
+      <c r="T10" s="86"/>
+      <c r="U10" s="86"/>
+      <c r="V10" s="86"/>
+      <c r="W10" s="86"/>
+      <c r="X10" s="86"/>
+      <c r="Y10" s="86"/>
+      <c r="Z10" s="86"/>
+      <c r="AA10" s="86"/>
+      <c r="AB10" s="86"/>
+      <c r="AC10" s="86"/>
+      <c r="AD10" s="86"/>
+      <c r="AE10" s="86"/>
+      <c r="AF10" s="86"/>
+      <c r="AG10" s="86"/>
+      <c r="AH10" s="86"/>
+      <c r="AI10" s="86"/>
+      <c r="AJ10" s="86"/>
+      <c r="AK10" s="86"/>
+      <c r="AL10" s="86"/>
+      <c r="AM10" s="86"/>
+      <c r="AN10" s="86"/>
+      <c r="AO10" s="86"/>
+      <c r="AP10" s="86"/>
+      <c r="AQ10" s="86"/>
+      <c r="AR10" s="86"/>
+      <c r="AS10" s="86"/>
+      <c r="AT10" s="86"/>
+      <c r="AU10" s="86"/>
+      <c r="AV10" s="87"/>
       <c r="BH10" s="4"/>
       <c r="BI10" s="4"/>
       <c r="BJ10" s="4"/>
@@ -2559,259 +2559,259 @@
       <c r="EJ10" s="4"/>
     </row>
     <row r="11" spans="1:140" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="88" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="51" t="s">
+      <c r="B11" s="89"/>
+      <c r="C11" s="89"/>
+      <c r="D11" s="89"/>
+      <c r="E11" s="89"/>
+      <c r="F11" s="89"/>
+      <c r="G11" s="90"/>
+      <c r="H11" s="91" t="s">
         <v>32</v>
       </c>
-      <c r="I11" s="21"/>
-      <c r="J11" s="21"/>
-      <c r="K11" s="21"/>
-      <c r="L11" s="21"/>
-      <c r="M11" s="21"/>
-      <c r="N11" s="21"/>
-      <c r="O11" s="21"/>
-      <c r="P11" s="22"/>
-      <c r="Q11" s="51" t="s">
+      <c r="I11" s="92"/>
+      <c r="J11" s="92"/>
+      <c r="K11" s="92"/>
+      <c r="L11" s="92"/>
+      <c r="M11" s="92"/>
+      <c r="N11" s="92"/>
+      <c r="O11" s="92"/>
+      <c r="P11" s="93"/>
+      <c r="Q11" s="91" t="s">
         <v>35</v>
       </c>
-      <c r="R11" s="21"/>
-      <c r="S11" s="21"/>
-      <c r="T11" s="21"/>
-      <c r="U11" s="21"/>
-      <c r="V11" s="21"/>
-      <c r="W11" s="21"/>
-      <c r="X11" s="21"/>
-      <c r="Y11" s="21"/>
-      <c r="Z11" s="21"/>
-      <c r="AA11" s="22"/>
-      <c r="AB11" s="51" t="s">
+      <c r="R11" s="92"/>
+      <c r="S11" s="92"/>
+      <c r="T11" s="92"/>
+      <c r="U11" s="92"/>
+      <c r="V11" s="92"/>
+      <c r="W11" s="92"/>
+      <c r="X11" s="92"/>
+      <c r="Y11" s="92"/>
+      <c r="Z11" s="92"/>
+      <c r="AA11" s="93"/>
+      <c r="AB11" s="91" t="s">
         <v>36</v>
       </c>
-      <c r="AC11" s="21"/>
-      <c r="AD11" s="21"/>
-      <c r="AE11" s="21"/>
-      <c r="AF11" s="21"/>
-      <c r="AG11" s="21"/>
-      <c r="AH11" s="21"/>
-      <c r="AI11" s="21"/>
-      <c r="AJ11" s="21"/>
-      <c r="AK11" s="22"/>
-      <c r="AL11" s="28"/>
-      <c r="AM11" s="29"/>
-      <c r="AN11" s="29"/>
-      <c r="AO11" s="29"/>
-      <c r="AP11" s="29"/>
-      <c r="AQ11" s="29"/>
-      <c r="AR11" s="29"/>
-      <c r="AS11" s="29"/>
-      <c r="AT11" s="29"/>
-      <c r="AU11" s="29"/>
-      <c r="AV11" s="30"/>
+      <c r="AC11" s="92"/>
+      <c r="AD11" s="92"/>
+      <c r="AE11" s="92"/>
+      <c r="AF11" s="92"/>
+      <c r="AG11" s="92"/>
+      <c r="AH11" s="92"/>
+      <c r="AI11" s="92"/>
+      <c r="AJ11" s="92"/>
+      <c r="AK11" s="93"/>
+      <c r="AL11" s="94"/>
+      <c r="AM11" s="95"/>
+      <c r="AN11" s="95"/>
+      <c r="AO11" s="95"/>
+      <c r="AP11" s="95"/>
+      <c r="AQ11" s="95"/>
+      <c r="AR11" s="95"/>
+      <c r="AS11" s="95"/>
+      <c r="AT11" s="95"/>
+      <c r="AU11" s="95"/>
+      <c r="AV11" s="96"/>
     </row>
     <row r="12" spans="1:140" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="48" t="s">
+      <c r="A12" s="101" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="49"/>
-      <c r="C12" s="49"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="49"/>
-      <c r="F12" s="49"/>
-      <c r="G12" s="50"/>
-      <c r="H12" s="51"/>
-      <c r="I12" s="21"/>
-      <c r="J12" s="21"/>
-      <c r="K12" s="21"/>
-      <c r="L12" s="21"/>
-      <c r="M12" s="21"/>
-      <c r="N12" s="21"/>
-      <c r="O12" s="21"/>
-      <c r="P12" s="22"/>
-      <c r="Q12" s="52"/>
-      <c r="R12" s="21"/>
-      <c r="S12" s="21"/>
-      <c r="T12" s="21"/>
-      <c r="U12" s="21"/>
-      <c r="V12" s="21"/>
-      <c r="W12" s="21"/>
-      <c r="X12" s="21"/>
-      <c r="Y12" s="21"/>
-      <c r="Z12" s="21"/>
-      <c r="AA12" s="22"/>
-      <c r="AB12" s="52"/>
-      <c r="AC12" s="53"/>
-      <c r="AD12" s="53"/>
-      <c r="AE12" s="53"/>
-      <c r="AF12" s="53"/>
-      <c r="AG12" s="53"/>
-      <c r="AH12" s="53"/>
-      <c r="AI12" s="53"/>
-      <c r="AJ12" s="53"/>
-      <c r="AK12" s="54"/>
-      <c r="AL12" s="28"/>
-      <c r="AM12" s="29"/>
-      <c r="AN12" s="29"/>
-      <c r="AO12" s="29"/>
-      <c r="AP12" s="29"/>
-      <c r="AQ12" s="29"/>
-      <c r="AR12" s="29"/>
-      <c r="AS12" s="29"/>
-      <c r="AT12" s="29"/>
-      <c r="AU12" s="29"/>
-      <c r="AV12" s="30"/>
+      <c r="B12" s="102"/>
+      <c r="C12" s="102"/>
+      <c r="D12" s="102"/>
+      <c r="E12" s="102"/>
+      <c r="F12" s="102"/>
+      <c r="G12" s="103"/>
+      <c r="H12" s="91"/>
+      <c r="I12" s="92"/>
+      <c r="J12" s="92"/>
+      <c r="K12" s="92"/>
+      <c r="L12" s="92"/>
+      <c r="M12" s="92"/>
+      <c r="N12" s="92"/>
+      <c r="O12" s="92"/>
+      <c r="P12" s="93"/>
+      <c r="Q12" s="110"/>
+      <c r="R12" s="92"/>
+      <c r="S12" s="92"/>
+      <c r="T12" s="92"/>
+      <c r="U12" s="92"/>
+      <c r="V12" s="92"/>
+      <c r="W12" s="92"/>
+      <c r="X12" s="92"/>
+      <c r="Y12" s="92"/>
+      <c r="Z12" s="92"/>
+      <c r="AA12" s="93"/>
+      <c r="AB12" s="110"/>
+      <c r="AC12" s="111"/>
+      <c r="AD12" s="111"/>
+      <c r="AE12" s="111"/>
+      <c r="AF12" s="111"/>
+      <c r="AG12" s="111"/>
+      <c r="AH12" s="111"/>
+      <c r="AI12" s="111"/>
+      <c r="AJ12" s="111"/>
+      <c r="AK12" s="112"/>
+      <c r="AL12" s="94"/>
+      <c r="AM12" s="95"/>
+      <c r="AN12" s="95"/>
+      <c r="AO12" s="95"/>
+      <c r="AP12" s="95"/>
+      <c r="AQ12" s="95"/>
+      <c r="AR12" s="95"/>
+      <c r="AS12" s="95"/>
+      <c r="AT12" s="95"/>
+      <c r="AU12" s="95"/>
+      <c r="AV12" s="96"/>
     </row>
     <row r="13" spans="1:140" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="48" t="s">
+      <c r="A13" s="101" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="49"/>
-      <c r="C13" s="49"/>
-      <c r="D13" s="49"/>
-      <c r="E13" s="49"/>
-      <c r="F13" s="49"/>
-      <c r="G13" s="50"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="21"/>
-      <c r="J13" s="21"/>
-      <c r="K13" s="21"/>
-      <c r="L13" s="21"/>
-      <c r="M13" s="21"/>
-      <c r="N13" s="21"/>
-      <c r="O13" s="21"/>
-      <c r="P13" s="22"/>
-      <c r="Q13" s="20"/>
-      <c r="R13" s="23"/>
-      <c r="S13" s="23"/>
-      <c r="T13" s="23"/>
-      <c r="U13" s="23"/>
-      <c r="V13" s="23"/>
-      <c r="W13" s="23"/>
-      <c r="X13" s="23"/>
-      <c r="Y13" s="23"/>
-      <c r="Z13" s="23"/>
-      <c r="AA13" s="24"/>
-      <c r="AB13" s="25"/>
-      <c r="AC13" s="26"/>
-      <c r="AD13" s="26"/>
-      <c r="AE13" s="26"/>
-      <c r="AF13" s="26"/>
-      <c r="AG13" s="26"/>
-      <c r="AH13" s="26"/>
-      <c r="AI13" s="26"/>
-      <c r="AJ13" s="26"/>
-      <c r="AK13" s="27"/>
-      <c r="AL13" s="28"/>
-      <c r="AM13" s="29"/>
-      <c r="AN13" s="29"/>
-      <c r="AO13" s="29"/>
-      <c r="AP13" s="29"/>
-      <c r="AQ13" s="29"/>
-      <c r="AR13" s="29"/>
-      <c r="AS13" s="29"/>
-      <c r="AT13" s="29"/>
-      <c r="AU13" s="29"/>
-      <c r="AV13" s="30"/>
+      <c r="B13" s="102"/>
+      <c r="C13" s="102"/>
+      <c r="D13" s="102"/>
+      <c r="E13" s="102"/>
+      <c r="F13" s="102"/>
+      <c r="G13" s="103"/>
+      <c r="H13" s="104"/>
+      <c r="I13" s="92"/>
+      <c r="J13" s="92"/>
+      <c r="K13" s="92"/>
+      <c r="L13" s="92"/>
+      <c r="M13" s="92"/>
+      <c r="N13" s="92"/>
+      <c r="O13" s="92"/>
+      <c r="P13" s="93"/>
+      <c r="Q13" s="104"/>
+      <c r="R13" s="105"/>
+      <c r="S13" s="105"/>
+      <c r="T13" s="105"/>
+      <c r="U13" s="105"/>
+      <c r="V13" s="105"/>
+      <c r="W13" s="105"/>
+      <c r="X13" s="105"/>
+      <c r="Y13" s="105"/>
+      <c r="Z13" s="105"/>
+      <c r="AA13" s="106"/>
+      <c r="AB13" s="107"/>
+      <c r="AC13" s="108"/>
+      <c r="AD13" s="108"/>
+      <c r="AE13" s="108"/>
+      <c r="AF13" s="108"/>
+      <c r="AG13" s="108"/>
+      <c r="AH13" s="108"/>
+      <c r="AI13" s="108"/>
+      <c r="AJ13" s="108"/>
+      <c r="AK13" s="109"/>
+      <c r="AL13" s="94"/>
+      <c r="AM13" s="95"/>
+      <c r="AN13" s="95"/>
+      <c r="AO13" s="95"/>
+      <c r="AP13" s="95"/>
+      <c r="AQ13" s="95"/>
+      <c r="AR13" s="95"/>
+      <c r="AS13" s="95"/>
+      <c r="AT13" s="95"/>
+      <c r="AU13" s="95"/>
+      <c r="AV13" s="96"/>
     </row>
     <row r="14" spans="1:140" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="88" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="21"/>
-      <c r="J14" s="21"/>
-      <c r="K14" s="21"/>
-      <c r="L14" s="21"/>
-      <c r="M14" s="21"/>
-      <c r="N14" s="21"/>
-      <c r="O14" s="21"/>
-      <c r="P14" s="22"/>
-      <c r="Q14" s="20"/>
-      <c r="R14" s="23"/>
-      <c r="S14" s="23"/>
-      <c r="T14" s="23"/>
-      <c r="U14" s="23"/>
-      <c r="V14" s="23"/>
-      <c r="W14" s="23"/>
-      <c r="X14" s="23"/>
-      <c r="Y14" s="23"/>
-      <c r="Z14" s="23"/>
-      <c r="AA14" s="24"/>
-      <c r="AB14" s="25"/>
-      <c r="AC14" s="26"/>
-      <c r="AD14" s="26"/>
-      <c r="AE14" s="26"/>
-      <c r="AF14" s="26"/>
-      <c r="AG14" s="26"/>
-      <c r="AH14" s="26"/>
-      <c r="AI14" s="26"/>
-      <c r="AJ14" s="26"/>
-      <c r="AK14" s="27"/>
-      <c r="AL14" s="28"/>
-      <c r="AM14" s="29"/>
-      <c r="AN14" s="29"/>
-      <c r="AO14" s="29"/>
-      <c r="AP14" s="29"/>
-      <c r="AQ14" s="29"/>
-      <c r="AR14" s="29"/>
-      <c r="AS14" s="29"/>
-      <c r="AT14" s="29"/>
-      <c r="AU14" s="29"/>
-      <c r="AV14" s="30"/>
+      <c r="B14" s="89"/>
+      <c r="C14" s="89"/>
+      <c r="D14" s="89"/>
+      <c r="E14" s="89"/>
+      <c r="F14" s="89"/>
+      <c r="G14" s="90"/>
+      <c r="H14" s="104"/>
+      <c r="I14" s="92"/>
+      <c r="J14" s="92"/>
+      <c r="K14" s="92"/>
+      <c r="L14" s="92"/>
+      <c r="M14" s="92"/>
+      <c r="N14" s="92"/>
+      <c r="O14" s="92"/>
+      <c r="P14" s="93"/>
+      <c r="Q14" s="104"/>
+      <c r="R14" s="105"/>
+      <c r="S14" s="105"/>
+      <c r="T14" s="105"/>
+      <c r="U14" s="105"/>
+      <c r="V14" s="105"/>
+      <c r="W14" s="105"/>
+      <c r="X14" s="105"/>
+      <c r="Y14" s="105"/>
+      <c r="Z14" s="105"/>
+      <c r="AA14" s="106"/>
+      <c r="AB14" s="107"/>
+      <c r="AC14" s="108"/>
+      <c r="AD14" s="108"/>
+      <c r="AE14" s="108"/>
+      <c r="AF14" s="108"/>
+      <c r="AG14" s="108"/>
+      <c r="AH14" s="108"/>
+      <c r="AI14" s="108"/>
+      <c r="AJ14" s="108"/>
+      <c r="AK14" s="109"/>
+      <c r="AL14" s="94"/>
+      <c r="AM14" s="95"/>
+      <c r="AN14" s="95"/>
+      <c r="AO14" s="95"/>
+      <c r="AP14" s="95"/>
+      <c r="AQ14" s="95"/>
+      <c r="AR14" s="95"/>
+      <c r="AS14" s="95"/>
+      <c r="AT14" s="95"/>
+      <c r="AU14" s="95"/>
+      <c r="AV14" s="96"/>
     </row>
     <row r="15" spans="1:140" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="31" t="s">
+      <c r="A15" s="114" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="32"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="32"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="39" t="s">
+      <c r="B15" s="115"/>
+      <c r="C15" s="115"/>
+      <c r="D15" s="115"/>
+      <c r="E15" s="115"/>
+      <c r="F15" s="115"/>
+      <c r="G15" s="116"/>
+      <c r="H15" s="123" t="s">
         <v>23</v>
       </c>
-      <c r="I15" s="39"/>
-      <c r="J15" s="39"/>
-      <c r="K15" s="39"/>
-      <c r="L15" s="39"/>
-      <c r="M15" s="39"/>
-      <c r="N15" s="39"/>
-      <c r="O15" s="39"/>
-      <c r="P15" s="39"/>
-      <c r="Q15" s="39"/>
-      <c r="R15" s="39"/>
-      <c r="S15" s="39"/>
-      <c r="T15" s="39"/>
-      <c r="U15" s="39"/>
-      <c r="V15" s="39"/>
-      <c r="W15" s="39"/>
-      <c r="X15" s="40"/>
-      <c r="Y15" s="41" t="s">
+      <c r="I15" s="123"/>
+      <c r="J15" s="123"/>
+      <c r="K15" s="123"/>
+      <c r="L15" s="123"/>
+      <c r="M15" s="123"/>
+      <c r="N15" s="123"/>
+      <c r="O15" s="123"/>
+      <c r="P15" s="123"/>
+      <c r="Q15" s="123"/>
+      <c r="R15" s="123"/>
+      <c r="S15" s="123"/>
+      <c r="T15" s="123"/>
+      <c r="U15" s="123"/>
+      <c r="V15" s="123"/>
+      <c r="W15" s="123"/>
+      <c r="X15" s="124"/>
+      <c r="Y15" s="125" t="s">
         <v>24</v>
       </c>
-      <c r="Z15" s="42"/>
-      <c r="AA15" s="42"/>
-      <c r="AB15" s="42"/>
-      <c r="AC15" s="42"/>
-      <c r="AD15" s="42"/>
-      <c r="AE15" s="42"/>
-      <c r="AF15" s="42"/>
-      <c r="AG15" s="43"/>
+      <c r="Z15" s="126"/>
+      <c r="AA15" s="126"/>
+      <c r="AB15" s="126"/>
+      <c r="AC15" s="126"/>
+      <c r="AD15" s="126"/>
+      <c r="AE15" s="126"/>
+      <c r="AF15" s="126"/>
+      <c r="AG15" s="127"/>
       <c r="AH15" s="7" t="s">
         <v>26</v>
       </c>
@@ -2831,205 +2831,205 @@
       <c r="AV15" s="8"/>
     </row>
     <row r="16" spans="1:140" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="34"/>
-      <c r="B16" s="128"/>
-      <c r="C16" s="128"/>
-      <c r="D16" s="128"/>
-      <c r="E16" s="128"/>
-      <c r="F16" s="128"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="129" t="s">
+      <c r="A16" s="117"/>
+      <c r="B16" s="118"/>
+      <c r="C16" s="118"/>
+      <c r="D16" s="118"/>
+      <c r="E16" s="118"/>
+      <c r="F16" s="118"/>
+      <c r="G16" s="119"/>
+      <c r="H16" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="I16" s="129"/>
-      <c r="J16" s="129"/>
-      <c r="K16" s="129"/>
-      <c r="L16" s="129"/>
-      <c r="M16" s="129"/>
-      <c r="N16" s="129"/>
-      <c r="O16" s="129"/>
-      <c r="P16" s="129"/>
-      <c r="Q16" s="129"/>
-      <c r="R16" s="129"/>
-      <c r="S16" s="129"/>
-      <c r="T16" s="129"/>
-      <c r="U16" s="129"/>
-      <c r="V16" s="129"/>
-      <c r="W16" s="129"/>
+      <c r="I16" s="18"/>
+      <c r="J16" s="18"/>
+      <c r="K16" s="18"/>
+      <c r="L16" s="18"/>
+      <c r="M16" s="18"/>
+      <c r="N16" s="18"/>
+      <c r="O16" s="18"/>
+      <c r="P16" s="18"/>
+      <c r="Q16" s="18"/>
+      <c r="R16" s="18"/>
+      <c r="S16" s="18"/>
+      <c r="T16" s="18"/>
+      <c r="U16" s="18"/>
+      <c r="V16" s="18"/>
+      <c r="W16" s="18"/>
       <c r="X16" s="9"/>
-      <c r="Y16" s="44"/>
-      <c r="Z16" s="130"/>
-      <c r="AA16" s="130"/>
-      <c r="AB16" s="130"/>
-      <c r="AC16" s="130"/>
-      <c r="AD16" s="130"/>
-      <c r="AE16" s="130"/>
-      <c r="AF16" s="130"/>
-      <c r="AG16" s="45"/>
-      <c r="AH16" s="129" t="s">
+      <c r="Y16" s="128"/>
+      <c r="Z16" s="129"/>
+      <c r="AA16" s="129"/>
+      <c r="AB16" s="129"/>
+      <c r="AC16" s="129"/>
+      <c r="AD16" s="129"/>
+      <c r="AE16" s="129"/>
+      <c r="AF16" s="129"/>
+      <c r="AG16" s="130"/>
+      <c r="AH16" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="AI16" s="129"/>
-      <c r="AJ16" s="129"/>
-      <c r="AK16" s="129"/>
-      <c r="AL16" s="129"/>
-      <c r="AM16" s="129"/>
-      <c r="AN16" s="129"/>
-      <c r="AO16" s="129"/>
-      <c r="AP16" s="129"/>
-      <c r="AQ16" s="129"/>
-      <c r="AR16" s="129"/>
-      <c r="AS16" s="129"/>
-      <c r="AT16" s="129"/>
-      <c r="AU16" s="129"/>
+      <c r="AI16" s="18"/>
+      <c r="AJ16" s="18"/>
+      <c r="AK16" s="18"/>
+      <c r="AL16" s="18"/>
+      <c r="AM16" s="18"/>
+      <c r="AN16" s="18"/>
+      <c r="AO16" s="18"/>
+      <c r="AP16" s="18"/>
+      <c r="AQ16" s="18"/>
+      <c r="AR16" s="18"/>
+      <c r="AS16" s="18"/>
+      <c r="AT16" s="18"/>
+      <c r="AU16" s="18"/>
       <c r="AV16" s="10"/>
     </row>
     <row r="17" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="34"/>
-      <c r="B17" s="128"/>
-      <c r="C17" s="128"/>
-      <c r="D17" s="128"/>
-      <c r="E17" s="128"/>
-      <c r="F17" s="128"/>
-      <c r="G17" s="35"/>
-      <c r="H17" s="129"/>
-      <c r="I17" s="129"/>
-      <c r="J17" s="129"/>
-      <c r="K17" s="129"/>
-      <c r="L17" s="129"/>
-      <c r="M17" s="129"/>
-      <c r="N17" s="129"/>
-      <c r="O17" s="129"/>
-      <c r="P17" s="129"/>
-      <c r="Q17" s="129"/>
-      <c r="R17" s="129"/>
-      <c r="S17" s="129"/>
-      <c r="T17" s="129"/>
-      <c r="U17" s="129"/>
-      <c r="V17" s="129"/>
-      <c r="W17" s="129"/>
+      <c r="A17" s="117"/>
+      <c r="B17" s="118"/>
+      <c r="C17" s="118"/>
+      <c r="D17" s="118"/>
+      <c r="E17" s="118"/>
+      <c r="F17" s="118"/>
+      <c r="G17" s="119"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="18"/>
+      <c r="L17" s="18"/>
+      <c r="M17" s="18"/>
+      <c r="N17" s="18"/>
+      <c r="O17" s="18"/>
+      <c r="P17" s="18"/>
+      <c r="Q17" s="18"/>
+      <c r="R17" s="18"/>
+      <c r="S17" s="18"/>
+      <c r="T17" s="18"/>
+      <c r="U17" s="18"/>
+      <c r="V17" s="18"/>
+      <c r="W17" s="18"/>
       <c r="X17" s="9"/>
-      <c r="Y17" s="44"/>
-      <c r="Z17" s="130"/>
-      <c r="AA17" s="130"/>
-      <c r="AB17" s="130"/>
-      <c r="AC17" s="130"/>
-      <c r="AD17" s="130"/>
-      <c r="AE17" s="130"/>
-      <c r="AF17" s="130"/>
-      <c r="AG17" s="45"/>
-      <c r="AH17" s="129"/>
-      <c r="AI17" s="129"/>
-      <c r="AJ17" s="129"/>
-      <c r="AK17" s="129"/>
-      <c r="AL17" s="129"/>
-      <c r="AM17" s="129"/>
-      <c r="AN17" s="129"/>
-      <c r="AO17" s="129"/>
-      <c r="AP17" s="129"/>
-      <c r="AQ17" s="129"/>
-      <c r="AR17" s="129"/>
-      <c r="AS17" s="129"/>
-      <c r="AT17" s="129"/>
-      <c r="AU17" s="129"/>
+      <c r="Y17" s="128"/>
+      <c r="Z17" s="129"/>
+      <c r="AA17" s="129"/>
+      <c r="AB17" s="129"/>
+      <c r="AC17" s="129"/>
+      <c r="AD17" s="129"/>
+      <c r="AE17" s="129"/>
+      <c r="AF17" s="129"/>
+      <c r="AG17" s="130"/>
+      <c r="AH17" s="18"/>
+      <c r="AI17" s="18"/>
+      <c r="AJ17" s="18"/>
+      <c r="AK17" s="18"/>
+      <c r="AL17" s="18"/>
+      <c r="AM17" s="18"/>
+      <c r="AN17" s="18"/>
+      <c r="AO17" s="18"/>
+      <c r="AP17" s="18"/>
+      <c r="AQ17" s="18"/>
+      <c r="AR17" s="18"/>
+      <c r="AS17" s="18"/>
+      <c r="AT17" s="18"/>
+      <c r="AU17" s="18"/>
       <c r="AV17" s="10"/>
     </row>
     <row r="18" spans="1:48" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="34"/>
-      <c r="B18" s="128"/>
-      <c r="C18" s="128"/>
-      <c r="D18" s="128"/>
-      <c r="E18" s="128"/>
-      <c r="F18" s="128"/>
-      <c r="G18" s="35"/>
+      <c r="A18" s="117"/>
+      <c r="B18" s="118"/>
+      <c r="C18" s="118"/>
+      <c r="D18" s="118"/>
+      <c r="E18" s="118"/>
+      <c r="F18" s="118"/>
+      <c r="G18" s="119"/>
       <c r="H18" s="11"/>
-      <c r="I18" s="131"/>
-      <c r="J18" s="132"/>
-      <c r="K18" s="132"/>
-      <c r="L18" s="130"/>
-      <c r="M18" s="130"/>
-      <c r="N18" s="130"/>
-      <c r="O18" s="130"/>
-      <c r="P18" s="130"/>
-      <c r="Q18" s="130"/>
-      <c r="R18" s="130"/>
-      <c r="S18" s="130"/>
-      <c r="T18" s="130"/>
-      <c r="U18" s="130"/>
-      <c r="V18" s="130"/>
-      <c r="W18" s="130"/>
-      <c r="X18" s="45"/>
-      <c r="Y18" s="44"/>
-      <c r="Z18" s="130"/>
-      <c r="AA18" s="130"/>
-      <c r="AB18" s="130"/>
-      <c r="AC18" s="130"/>
-      <c r="AD18" s="130"/>
-      <c r="AE18" s="130"/>
-      <c r="AF18" s="130"/>
-      <c r="AG18" s="45"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="20"/>
+      <c r="K18" s="20"/>
+      <c r="L18" s="129"/>
+      <c r="M18" s="129"/>
+      <c r="N18" s="129"/>
+      <c r="O18" s="129"/>
+      <c r="P18" s="129"/>
+      <c r="Q18" s="129"/>
+      <c r="R18" s="129"/>
+      <c r="S18" s="129"/>
+      <c r="T18" s="129"/>
+      <c r="U18" s="129"/>
+      <c r="V18" s="129"/>
+      <c r="W18" s="129"/>
+      <c r="X18" s="130"/>
+      <c r="Y18" s="128"/>
+      <c r="Z18" s="129"/>
+      <c r="AA18" s="129"/>
+      <c r="AB18" s="129"/>
+      <c r="AC18" s="129"/>
+      <c r="AD18" s="129"/>
+      <c r="AE18" s="129"/>
+      <c r="AF18" s="129"/>
+      <c r="AG18" s="130"/>
       <c r="AH18" s="11"/>
-      <c r="AI18" s="131"/>
-      <c r="AJ18" s="131"/>
-      <c r="AK18" s="131"/>
-      <c r="AL18" s="131"/>
-      <c r="AM18" s="131"/>
-      <c r="AN18" s="131"/>
-      <c r="AO18" s="131"/>
-      <c r="AP18" s="131"/>
-      <c r="AQ18" s="131"/>
-      <c r="AR18" s="131"/>
-      <c r="AS18" s="131"/>
-      <c r="AT18" s="131"/>
-      <c r="AU18" s="131"/>
+      <c r="AI18" s="19"/>
+      <c r="AJ18" s="19"/>
+      <c r="AK18" s="19"/>
+      <c r="AL18" s="19"/>
+      <c r="AM18" s="19"/>
+      <c r="AN18" s="19"/>
+      <c r="AO18" s="19"/>
+      <c r="AP18" s="19"/>
+      <c r="AQ18" s="19"/>
+      <c r="AR18" s="19"/>
+      <c r="AS18" s="19"/>
+      <c r="AT18" s="19"/>
+      <c r="AU18" s="19"/>
       <c r="AV18" s="12"/>
     </row>
     <row r="19" spans="1:48" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="36"/>
-      <c r="B19" s="37"/>
-      <c r="C19" s="37"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="37"/>
-      <c r="G19" s="38"/>
+      <c r="A19" s="120"/>
+      <c r="B19" s="121"/>
+      <c r="C19" s="121"/>
+      <c r="D19" s="121"/>
+      <c r="E19" s="121"/>
+      <c r="F19" s="121"/>
+      <c r="G19" s="122"/>
       <c r="H19" s="13"/>
       <c r="I19" s="13"/>
       <c r="J19" s="14"/>
       <c r="K19" s="14"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="16"/>
-      <c r="O19" s="16"/>
-      <c r="P19" s="16"/>
-      <c r="Q19" s="16"/>
-      <c r="R19" s="16"/>
-      <c r="S19" s="16"/>
-      <c r="T19" s="16"/>
-      <c r="U19" s="16"/>
-      <c r="V19" s="16"/>
-      <c r="W19" s="16"/>
-      <c r="X19" s="16"/>
-      <c r="Y19" s="46"/>
-      <c r="Z19" s="16"/>
-      <c r="AA19" s="16"/>
-      <c r="AB19" s="16"/>
-      <c r="AC19" s="16"/>
-      <c r="AD19" s="16"/>
-      <c r="AE19" s="16"/>
-      <c r="AF19" s="16"/>
-      <c r="AG19" s="47"/>
+      <c r="L19" s="113"/>
+      <c r="M19" s="113"/>
+      <c r="N19" s="113"/>
+      <c r="O19" s="113"/>
+      <c r="P19" s="113"/>
+      <c r="Q19" s="113"/>
+      <c r="R19" s="113"/>
+      <c r="S19" s="113"/>
+      <c r="T19" s="113"/>
+      <c r="U19" s="113"/>
+      <c r="V19" s="113"/>
+      <c r="W19" s="113"/>
+      <c r="X19" s="113"/>
+      <c r="Y19" s="131"/>
+      <c r="Z19" s="113"/>
+      <c r="AA19" s="113"/>
+      <c r="AB19" s="113"/>
+      <c r="AC19" s="113"/>
+      <c r="AD19" s="113"/>
+      <c r="AE19" s="113"/>
+      <c r="AF19" s="113"/>
+      <c r="AG19" s="132"/>
       <c r="AH19" s="13"/>
-      <c r="AI19" s="16"/>
-      <c r="AJ19" s="16"/>
-      <c r="AK19" s="16"/>
-      <c r="AL19" s="16"/>
-      <c r="AM19" s="16"/>
-      <c r="AN19" s="16"/>
-      <c r="AO19" s="16"/>
-      <c r="AP19" s="16"/>
-      <c r="AQ19" s="16"/>
-      <c r="AR19" s="16"/>
-      <c r="AS19" s="16"/>
+      <c r="AI19" s="113"/>
+      <c r="AJ19" s="113"/>
+      <c r="AK19" s="113"/>
+      <c r="AL19" s="113"/>
+      <c r="AM19" s="113"/>
+      <c r="AN19" s="113"/>
+      <c r="AO19" s="113"/>
+      <c r="AP19" s="113"/>
+      <c r="AQ19" s="113"/>
+      <c r="AR19" s="113"/>
+      <c r="AS19" s="113"/>
       <c r="AT19" s="13"/>
       <c r="AU19" s="13"/>
       <c r="AV19" s="15"/>
@@ -3058,28 +3058,39 @@
     <row r="41" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="71">
-    <mergeCell ref="W9:X9"/>
-    <mergeCell ref="Y9:AD9"/>
-    <mergeCell ref="AE9:AK9"/>
-    <mergeCell ref="AL9:AR9"/>
-    <mergeCell ref="AS9:AT9"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="H9:L9"/>
-    <mergeCell ref="M9:S9"/>
-    <mergeCell ref="T9:V9"/>
-    <mergeCell ref="A1:H5"/>
-    <mergeCell ref="I1:AK5"/>
-    <mergeCell ref="AL1:AR1"/>
-    <mergeCell ref="AS1:AV1"/>
-    <mergeCell ref="AL2:AR2"/>
-    <mergeCell ref="AS2:AV2"/>
-    <mergeCell ref="AL3:AR3"/>
-    <mergeCell ref="AS3:AV3"/>
-    <mergeCell ref="AL4:AR4"/>
-    <mergeCell ref="AS4:AV4"/>
-    <mergeCell ref="AL5:AR5"/>
-    <mergeCell ref="AS5:AV5"/>
+    <mergeCell ref="AI19:AS19"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="H14:P14"/>
+    <mergeCell ref="Q14:AA14"/>
+    <mergeCell ref="AB14:AK14"/>
+    <mergeCell ref="AL14:AV14"/>
+    <mergeCell ref="A15:G19"/>
+    <mergeCell ref="H15:X15"/>
+    <mergeCell ref="Y15:AG19"/>
+    <mergeCell ref="L18:X18"/>
+    <mergeCell ref="L19:X19"/>
+    <mergeCell ref="AL8:AR8"/>
+    <mergeCell ref="AL12:AV12"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="H13:P13"/>
+    <mergeCell ref="Q13:AA13"/>
+    <mergeCell ref="AB13:AK13"/>
+    <mergeCell ref="AL13:AV13"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="H12:P12"/>
+    <mergeCell ref="Q12:AA12"/>
+    <mergeCell ref="AB12:AK12"/>
+    <mergeCell ref="H8:L8"/>
+    <mergeCell ref="M8:S8"/>
+    <mergeCell ref="T8:V8"/>
+    <mergeCell ref="Y8:AD8"/>
+    <mergeCell ref="AE8:AK8"/>
+    <mergeCell ref="A10:AV10"/>
+    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="H11:P11"/>
+    <mergeCell ref="Q11:AA11"/>
+    <mergeCell ref="AB11:AK11"/>
+    <mergeCell ref="AL11:AV11"/>
     <mergeCell ref="AS8:AT8"/>
     <mergeCell ref="AL7:AV7"/>
     <mergeCell ref="A6:F6"/>
@@ -3094,41 +3105,30 @@
     <mergeCell ref="AG7:AK7"/>
     <mergeCell ref="AL6:AV6"/>
     <mergeCell ref="W8:X8"/>
-    <mergeCell ref="A10:AV10"/>
-    <mergeCell ref="A11:G11"/>
-    <mergeCell ref="H11:P11"/>
-    <mergeCell ref="Q11:AA11"/>
-    <mergeCell ref="AB11:AK11"/>
-    <mergeCell ref="AL11:AV11"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C8:G8"/>
-    <mergeCell ref="H8:L8"/>
-    <mergeCell ref="M8:S8"/>
-    <mergeCell ref="T8:V8"/>
-    <mergeCell ref="Y8:AD8"/>
-    <mergeCell ref="AE8:AK8"/>
-    <mergeCell ref="AL8:AR8"/>
-    <mergeCell ref="AL12:AV12"/>
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="H13:P13"/>
-    <mergeCell ref="Q13:AA13"/>
-    <mergeCell ref="AB13:AK13"/>
-    <mergeCell ref="AL13:AV13"/>
-    <mergeCell ref="A12:G12"/>
-    <mergeCell ref="H12:P12"/>
-    <mergeCell ref="Q12:AA12"/>
-    <mergeCell ref="AB12:AK12"/>
-    <mergeCell ref="AI19:AS19"/>
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="H14:P14"/>
-    <mergeCell ref="Q14:AA14"/>
-    <mergeCell ref="AB14:AK14"/>
-    <mergeCell ref="AL14:AV14"/>
-    <mergeCell ref="A15:G19"/>
-    <mergeCell ref="H15:X15"/>
-    <mergeCell ref="Y15:AG19"/>
-    <mergeCell ref="L18:X18"/>
-    <mergeCell ref="L19:X19"/>
+    <mergeCell ref="A1:H5"/>
+    <mergeCell ref="I1:AK5"/>
+    <mergeCell ref="AL1:AR1"/>
+    <mergeCell ref="AS1:AV1"/>
+    <mergeCell ref="AL2:AR2"/>
+    <mergeCell ref="AS2:AV2"/>
+    <mergeCell ref="AL3:AR3"/>
+    <mergeCell ref="AS3:AV3"/>
+    <mergeCell ref="AL4:AR4"/>
+    <mergeCell ref="AS4:AV4"/>
+    <mergeCell ref="AL5:AR5"/>
+    <mergeCell ref="AS5:AV5"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="H9:L9"/>
+    <mergeCell ref="M9:S9"/>
+    <mergeCell ref="T9:V9"/>
+    <mergeCell ref="W9:X9"/>
+    <mergeCell ref="Y9:AD9"/>
+    <mergeCell ref="AE9:AK9"/>
+    <mergeCell ref="AL9:AR9"/>
+    <mergeCell ref="AS9:AT9"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>